<commit_message>
Aplica auditoria de taxonomia e publica triagem de cedentes
</commit_message>
<xml_diff>
--- a/data/industry_study/generated_revision/top100_fidcs_middle_market.xlsx
+++ b/data/industry_study/generated_revision/top100_fidcs_middle_market.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" r:id="R3b9c20ba1fe94ba7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 100 FIDCs" sheetId="2" r:id="R074fbef911d6446b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" r:id="Rb7e630a415f442dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 100 FIDCs" sheetId="2" r:id="R82f93c5d356541fc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1180,16 +1180,16 @@
         <x:v>Recebíveis Comerciais</x:v>
       </x:c>
       <x:c r="AA7" s="23" t="str">
-        <x:v>Agro, Indústria e Comércio</x:v>
+        <x:v>Outros</x:v>
       </x:c>
       <x:c r="AB7" s="23" t="str">
-        <x:v>Recebíveis Comerciais</x:v>
+        <x:v>Multicedente/Multissacado</x:v>
       </x:c>
       <x:c r="AC7" s="23" t="str">
-        <x:v>N/D</x:v>
+        <x:v>Crédito PF</x:v>
       </x:c>
       <x:c r="AD7" s="23" t="str">
-        <x:v>N/D</x:v>
+        <x:v>Auto/Veículos</x:v>
       </x:c>
       <x:c r="AE7" s="27" t="b">
         <x:v>0</x:v>
@@ -1213,7 +1213,7 @@
         <x:v>N/D</x:v>
       </x:c>
       <x:c r="AL7" s="23" t="str">
-        <x:v>N/D</x:v>
+        <x:v>IME 03 a 06/2026, blocos SEGMT, COMPMT_DICRED_SEM_AQUIS e PRAZO_VENC; DF de cisao 18/03/2026, balanco patrimonial</x:v>
       </x:c>
       <x:c r="AM7" s="23" t="str">
         <x:v>N/D</x:v>
@@ -2558,7 +2558,7 @@
         <x:v>Financeiro</x:v>
       </x:c>
       <x:c r="AB18" s="24" t="str">
-        <x:v>Crédito PF</x:v>
+        <x:v>Multicarteira Financeiro</x:v>
       </x:c>
       <x:c r="AC18" s="24" t="str">
         <x:v>Crédito PF</x:v>
@@ -2930,10 +2930,10 @@
         <x:v>Financiamento de Veículos</x:v>
       </x:c>
       <x:c r="AA21" s="23" t="str">
-        <x:v>Financeiro</x:v>
+        <x:v>Agro, Indústria e Comércio</x:v>
       </x:c>
       <x:c r="AB21" s="23" t="str">
-        <x:v>Financiamento de Veículos</x:v>
+        <x:v>Recebíveis Comerciais</x:v>
       </x:c>
       <x:c r="AC21" s="23" t="str">
         <x:v>Crédito PF</x:v>
@@ -3558,7 +3558,7 @@
         <x:v>Outros</x:v>
       </x:c>
       <x:c r="AB26" s="24" t="str">
-        <x:v>Poder Público</x:v>
+        <x:v>Recuperação</x:v>
       </x:c>
       <x:c r="AC26" s="24" t="str">
         <x:v>Judicial/Precatórios/NPL</x:v>
@@ -3582,7 +3582,7 @@
         <x:v>Comentário manual do usuário — IMG_8592.jpg</x:v>
       </x:c>
       <x:c r="AJ26" s="24" t="str">
-        <x:v>IMG_8592</x:v>
+        <x:v>Regulamento ids 762766 e 762773</x:v>
       </x:c>
       <x:c r="AK26" s="24" t="str">
         <x:v>N/D</x:v>
@@ -3680,10 +3680,10 @@
         <x:v>Multicarteira Outros</x:v>
       </x:c>
       <x:c r="AA27" s="23" t="str">
-        <x:v>Outros</x:v>
+        <x:v>Agro, Indústria e Comércio</x:v>
       </x:c>
       <x:c r="AB27" s="23" t="str">
-        <x:v>Multicarteira Outros</x:v>
+        <x:v>Crédito Corporativo</x:v>
       </x:c>
       <x:c r="AC27" s="23" t="str">
         <x:v>Multissetorial / Outros</x:v>
@@ -3805,10 +3805,10 @@
         <x:v>Multicarteira Outros</x:v>
       </x:c>
       <x:c r="AA28" s="24" t="str">
-        <x:v>Fomento Mercantil</x:v>
+        <x:v>Outros</x:v>
       </x:c>
       <x:c r="AB28" s="24" t="str">
-        <x:v>Fomento Mercantil</x:v>
+        <x:v>Recuperação</x:v>
       </x:c>
       <x:c r="AC28" s="24" t="str">
         <x:v>Crédito PJ</x:v>
@@ -3832,7 +3832,7 @@
         <x:v>Comentário manual do usuário — IMG_8592.jpg</x:v>
       </x:c>
       <x:c r="AJ28" s="24" t="str">
-        <x:v>IMG_8592</x:v>
+        <x:v>Regulamento arquivado no FundosNET</x:v>
       </x:c>
       <x:c r="AK28" s="24" t="str">
         <x:v>N/D</x:v>
@@ -4305,10 +4305,10 @@
         <x:v>Fomento Mercantil</x:v>
       </x:c>
       <x:c r="AA32" s="24" t="str">
-        <x:v>Fomento Mercantil</x:v>
+        <x:v>Agro, Indústria e Comércio</x:v>
       </x:c>
       <x:c r="AB32" s="24" t="str">
-        <x:v>Fomento Mercantil</x:v>
+        <x:v>Crédito Corporativo</x:v>
       </x:c>
       <x:c r="AC32" s="24" t="str">
         <x:v>Crédito PJ</x:v>
@@ -4332,7 +4332,7 @@
         <x:v>https://fnet.bmfbovespa.com.br/fnet/publico/abrirGerenciadorDocumentosCVM?cnpjFundo=62393829000159</x:v>
       </x:c>
       <x:c r="AJ32" s="24" t="str">
-        <x:v>1242436</x:v>
+        <x:v>Regulamento id 1231073 e correlatos</x:v>
       </x:c>
       <x:c r="AK32" s="24" t="str">
         <x:v>N/D</x:v>
@@ -4808,7 +4808,7 @@
         <x:v>Outros</x:v>
       </x:c>
       <x:c r="AB36" s="24" t="str">
-        <x:v>Multicarteira Outros</x:v>
+        <x:v>Recuperação</x:v>
       </x:c>
       <x:c r="AC36" s="24" t="str">
         <x:v>Multissetorial / Outros</x:v>
@@ -4832,7 +4832,7 @@
         <x:v>https://fnet.bmfbovespa.com.br/fnet/publico/abrirGerenciadorDocumentosCVM?cnpjFundo=51079269000146</x:v>
       </x:c>
       <x:c r="AJ36" s="24" t="str">
-        <x:v>884671</x:v>
+        <x:v>Regulamento id 884671</x:v>
       </x:c>
       <x:c r="AK36" s="24" t="str">
         <x:v>N/D</x:v>
@@ -5582,7 +5582,7 @@
         <x:v>Comentário explícito do usuário — tarefa Adquirência</x:v>
       </x:c>
       <x:c r="AJ42" s="24" t="str">
-        <x:v>chat_task_acquiring_2026_07_31</x:v>
+        <x:v>Regulamento arquivado no FundosNET</x:v>
       </x:c>
       <x:c r="AK42" s="24" t="str">
         <x:v>N/D</x:v>
@@ -5826,7 +5826,7 @@
         <x:v>A evidência disponível aponta outro tipo de risco ou não traz crédito corporativo.</x:v>
       </x:c>
       <x:c r="AH44" s="24" t="str">
-        <x:v>Financeiro → Adquirência; risco banco emissor</x:v>
+        <x:v>A CloudWalk é definida como cedente dos recebíveis de transações de pagamento devidos pelos emissores.</x:v>
       </x:c>
       <x:c r="AI44" s="24" t="str">
         <x:v>Comentário explícito do usuário — tarefa Adquirência</x:v>
@@ -6207,7 +6207,7 @@
         <x:v>https://fnet.bmfbovespa.com.br/fnet/publico/abrirGerenciadorDocumentosCVM?cnpjFundo=26405883000103</x:v>
       </x:c>
       <x:c r="AJ47" s="23" t="str">
-        <x:v>787165</x:v>
+        <x:v>Regulamento id 787165</x:v>
       </x:c>
       <x:c r="AK47" s="23" t="str">
         <x:v>N/D</x:v>
@@ -8546,7 +8546,7 @@
         <x:v>N/D</x:v>
       </x:c>
       <x:c r="X66" s="24" t="str">
-        <x:v>N/D</x:v>
+        <x:v>FGTS</x:v>
       </x:c>
       <x:c r="Y66" s="24" t="str">
         <x:v>Financeiro</x:v>
@@ -8558,37 +8558,37 @@
         <x:v>Financeiro</x:v>
       </x:c>
       <x:c r="AB66" s="24" t="str">
-        <x:v>Crédito Pessoal</x:v>
+        <x:v>Crédito Consignado</x:v>
       </x:c>
       <x:c r="AC66" s="24" t="str">
-        <x:v>N/D</x:v>
+        <x:v>Crédito PF</x:v>
       </x:c>
       <x:c r="AD66" s="24" t="str">
-        <x:v>N/D</x:v>
+        <x:v>FGTS</x:v>
       </x:c>
       <x:c r="AE66" s="24" t="str">
         <x:v>N/D</x:v>
       </x:c>
       <x:c r="AF66" s="24" t="str">
-        <x:v>N/D — dados insuficientes</x:v>
+        <x:v>Indício de crédito corporativo; porte N/D</x:v>
       </x:c>
       <x:c r="AG66" s="24" t="str">
-        <x:v>Cedente, sacado e tipo de recebível não foram localizados.</x:v>
+        <x:v>O lastro é compatível com crédito corporativo tradicional, mas a base não documenta o porte do tomador.</x:v>
       </x:c>
       <x:c r="AH66" s="24" t="str">
-        <x:v>N/D</x:v>
+        <x:v>Def. "Endossante": cada instituição financeira que ceda Direitos Creditórios à Classe. Def. "Devedores": cada trabalhador beneficiário do FGTS que emita CCB com cessão fiduciária do Saque-aniversário. A Tabela II aloca 100% em C1 "Comercial", campo incompatível com CCB de pessoa física garantida por FGTS.</x:v>
       </x:c>
       <x:c r="AI66" s="24" t="str">
-        <x:v>ANBIMA Data — Fundos 175: características público</x:v>
+        <x:v>Industria_FIDC_202606_auditada.xlsx#Auditoria classificação Top200</x:v>
       </x:c>
       <x:c r="AJ66" s="24" t="str">
-        <x:v>N/D</x:v>
+        <x:v>Regulamento ids 670689 e 670690</x:v>
       </x:c>
       <x:c r="AK66" s="24" t="str">
         <x:v>N/D</x:v>
       </x:c>
       <x:c r="AL66" s="24" t="str">
-        <x:v>N/D</x:v>
+        <x:v>Regulamento ids 670689 e 670690</x:v>
       </x:c>
       <x:c r="AM66" s="24" t="str">
         <x:v>N/D</x:v>
@@ -8597,7 +8597,7 @@
         <x:v>N/D</x:v>
       </x:c>
       <x:c r="AO66" s="24" t="str">
-        <x:v>N/D</x:v>
+        <x:v>taxonomia disponível — partes e lastro documental N/D</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="36" customHeight="1">
@@ -9832,7 +9832,7 @@
         <x:v>Comentário explícito do usuário — tarefa Adquirência</x:v>
       </x:c>
       <x:c r="AJ76" s="24" t="str">
-        <x:v>chat_task_acquiring_2026_07_31</x:v>
+        <x:v>Regulamento id 1091930 e correlatos</x:v>
       </x:c>
       <x:c r="AK76" s="24" t="str">
         <x:v>N/D</x:v>
@@ -10183,7 +10183,7 @@
         <x:v>Financeiro</x:v>
       </x:c>
       <x:c r="AB79" s="23" t="str">
-        <x:v>Cartão de crédito</x:v>
+        <x:v>Multicarteira Financeiro</x:v>
       </x:c>
       <x:c r="AC79" s="23" t="str">
         <x:v>Meios de Pagamento e Cartões</x:v>
@@ -10207,7 +10207,7 @@
         <x:v>FundosNet/B3 — regulamento 1186789</x:v>
       </x:c>
       <x:c r="AJ79" s="23" t="str">
-        <x:v>1186789</x:v>
+        <x:v>Regulamento id 1186789</x:v>
       </x:c>
       <x:c r="AK79" s="23" t="str">
         <x:v>N/D</x:v>
@@ -10433,7 +10433,7 @@
         <x:v>Financeiro</x:v>
       </x:c>
       <x:c r="AB81" s="23" t="str">
-        <x:v>Crédito Pessoal</x:v>
+        <x:v>Crédito Consignado</x:v>
       </x:c>
       <x:c r="AC81" s="23" t="str">
         <x:v>Multissetorial / Outros</x:v>
@@ -10933,7 +10933,7 @@
         <x:v>Financeiro</x:v>
       </x:c>
       <x:c r="AB85" s="23" t="str">
-        <x:v>Cartão de crédito</x:v>
+        <x:v>Multicarteira Financeiro</x:v>
       </x:c>
       <x:c r="AC85" s="23" t="str">
         <x:v>Meios de Pagamento e Cartões</x:v>
@@ -11796,7 +11796,7 @@
         <x:v>N/D</x:v>
       </x:c>
       <x:c r="X92" s="24" t="str">
-        <x:v>N/D</x:v>
+        <x:v>Auto/Veículos</x:v>
       </x:c>
       <x:c r="Y92" s="24" t="str">
         <x:v>Financeiro</x:v>
@@ -11808,37 +11808,37 @@
         <x:v>Financeiro</x:v>
       </x:c>
       <x:c r="AB92" s="24" t="str">
-        <x:v>Multicarteira Financeiro</x:v>
+        <x:v>Financiamento de Veículos</x:v>
       </x:c>
       <x:c r="AC92" s="24" t="str">
-        <x:v>N/D</x:v>
+        <x:v>Crédito PF</x:v>
       </x:c>
       <x:c r="AD92" s="24" t="str">
-        <x:v>N/D</x:v>
+        <x:v>Auto/Veículos</x:v>
       </x:c>
       <x:c r="AE92" s="24" t="str">
         <x:v>N/D</x:v>
       </x:c>
       <x:c r="AF92" s="24" t="str">
-        <x:v>N/D — dados insuficientes</x:v>
+        <x:v>Indício de crédito corporativo; porte N/D</x:v>
       </x:c>
       <x:c r="AG92" s="24" t="str">
-        <x:v>Cedente, sacado e tipo de recebível não foram localizados.</x:v>
+        <x:v>O lastro é compatível com crédito corporativo tradicional, mas a base não documenta o porte do tomador.</x:v>
       </x:c>
       <x:c r="AH92" s="24" t="str">
-        <x:v>N/D</x:v>
+        <x:v>Def. "Devedores": pessoas físicas que adquiriram um Veículo Automotor mediante financiamento concedido pelo Emitente por meio de emissão de CCBs. É financiamento ao consumidor, o oposto do floor plan de montadora.</x:v>
       </x:c>
       <x:c r="AI92" s="24" t="str">
-        <x:v>equivalência metodológica a partir do segmento CVM</x:v>
+        <x:v>Industria_FIDC_202606_auditada.xlsx#Auditoria classificação Top200</x:v>
       </x:c>
       <x:c r="AJ92" s="24" t="str">
-        <x:v>N/D</x:v>
+        <x:v>Regulamento arquivado no FundosNET</x:v>
       </x:c>
       <x:c r="AK92" s="24" t="str">
         <x:v>N/D</x:v>
       </x:c>
       <x:c r="AL92" s="24" t="str">
-        <x:v>N/D</x:v>
+        <x:v>Regulamento arquivado no FundosNET</x:v>
       </x:c>
       <x:c r="AM92" s="24" t="str">
         <x:v>N/D</x:v>
@@ -11847,7 +11847,7 @@
         <x:v>N/D</x:v>
       </x:c>
       <x:c r="AO92" s="24" t="str">
-        <x:v>N/D</x:v>
+        <x:v>taxonomia disponível — partes e lastro documental N/D</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="36" customHeight="1">
@@ -11957,7 +11957,7 @@
         <x:v>https://fnet.bmfbovespa.com.br/fnet/publico/abrirGerenciadorDocumentosCVM?cnpjFundo=39669950000149</x:v>
       </x:c>
       <x:c r="AJ93" s="23" t="str">
-        <x:v>1238679</x:v>
+        <x:v>Regulamento id 1238679</x:v>
       </x:c>
       <x:c r="AK93" s="23" t="str">
         <x:v>N/D</x:v>
@@ -12058,7 +12058,7 @@
         <x:v>Outros</x:v>
       </x:c>
       <x:c r="AB94" s="24" t="str">
-        <x:v>Poder Público</x:v>
+        <x:v>Recuperação</x:v>
       </x:c>
       <x:c r="AC94" s="24" t="str">
         <x:v>Judicial/Precatórios/NPL</x:v>
@@ -12082,7 +12082,7 @@
         <x:v>https://fnet.bmfbovespa.com.br/fnet/publico/abrirGerenciadorDocumentosCVM?cnpjFundo=13764696000174</x:v>
       </x:c>
       <x:c r="AJ94" s="24" t="str">
-        <x:v>734547</x:v>
+        <x:v>Regulamento id 734547</x:v>
       </x:c>
       <x:c r="AK94" s="24" t="str">
         <x:v>N/D</x:v>
@@ -12555,10 +12555,10 @@
         <x:v>Recebíveis Comerciais</x:v>
       </x:c>
       <x:c r="AA98" s="24" t="str">
-        <x:v>Agro, Indústria e Comércio</x:v>
+        <x:v>Financeiro</x:v>
       </x:c>
       <x:c r="AB98" s="24" t="str">
-        <x:v>Recebíveis Comerciais</x:v>
+        <x:v>Adquirência</x:v>
       </x:c>
       <x:c r="AC98" s="24" t="str">
         <x:v>Meios de Pagamento e Cartões</x:v>
@@ -12933,7 +12933,7 @@
         <x:v>Outros</x:v>
       </x:c>
       <x:c r="AB101" s="23" t="str">
-        <x:v>Poder Público</x:v>
+        <x:v>Recuperação</x:v>
       </x:c>
       <x:c r="AC101" s="23" t="str">
         <x:v>Judicial/Precatórios/NPL</x:v>
@@ -12957,7 +12957,7 @@
         <x:v>https://fnet.bmfbovespa.com.br/fnet/publico/abrirGerenciadorDocumentosCVM?cnpjFundo=45207707000101</x:v>
       </x:c>
       <x:c r="AJ101" s="23" t="str">
-        <x:v>779778</x:v>
+        <x:v>Regulamento id 779778</x:v>
       </x:c>
       <x:c r="AK101" s="23" t="str">
         <x:v>N/D</x:v>

</xml_diff>

<commit_message>
Corrige remuneração-alvo e enriquece rankings Top 15
</commit_message>
<xml_diff>
--- a/data/industry_study/generated_revision/top100_fidcs_middle_market.xlsx
+++ b/data/industry_study/generated_revision/top100_fidcs_middle_market.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" r:id="Rb7e630a415f442dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 100 FIDCs" sheetId="2" r:id="R82f93c5d356541fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" r:id="Rbdc9b91b8b9e4b91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 100 FIDCs" sheetId="2" r:id="Rcf9d4dfa11a643e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4326,7 +4326,7 @@
         <x:v>O lastro é compatível com crédito corporativo tradicional, mas a base não documenta o porte do tomador.</x:v>
       </x:c>
       <x:c r="AH32" s="24" t="str">
-        <x:v>Comentário manual do usuário — IMG_8706.JPG; planilha amarela; linha da raiz 62393829</x:v>
+        <x:v>INVESTIMENTO, DIVERSIFICACAO E COMPOSICAO DA CARTEIRA PREVISTAS NESTE CAPITULO SERAO OBSERVADAS DIARIAMENTE, COM BASE NO PATRIMONIO LIQUIDO DO DIA UTIL IMEDIATAMENTE ANTERIOR. 9. DIREITOS CREDITORIOS CARACTERISTICAS DOS DIREITOS CREDITORIOS OS DIREITOS CREDITORIOS A SEREM ADQUIRIDOS PELA CLASSE SAO DIREITOS CREDITORIOS PERFORMADOS, DECORRENTES DE OPERACOES DE COMPRA E VENDA DE PRODUTOS E PRESTACAO DE SERVICOS PELOS CEDENTES AS DEVEDORAS, REALIZADAS NO SEGMENTO COMERCIAL, BEM COMO RECEBIVEIS DE CARTAO DE CREDITO 9.1.1. A CLASSE NAO PODERA ADQUIRIR DIREITOS CREDITORIOS NAO PADRONIZADOS E/OU NAO PERFORMADOS, CUJA EXIGIBILIDADE AINDA DEPENDA DA CONTRAPRESTACAO PELOS RESPECTIVOS CEDENTES. 9.1.2. OS TERMOS DE CESSAO A SER EM FIRMADOS NA CESSAO DOS RECEBIVEIS DE CARTOES DE CREDITO COM CADA UMA DAS CREDENCIADORAS DEVERAO SER APRESENTADOS AOS COTISTAS SENIORES DE CADA SERIE INDIVIDUALMENTE ANTES DA FORMALIZACAO COM CADA CREDENC</x:v>
       </x:c>
       <x:c r="AI32" s="24" t="str">
         <x:v>https://fnet.bmfbovespa.com.br/fnet/publico/abrirGerenciadorDocumentosCVM?cnpjFundo=62393829000159</x:v>

</xml_diff>

<commit_message>
Melhora leitura dos rankings por tipo
</commit_message>
<xml_diff>
--- a/data/industry_study/generated_revision/top100_fidcs_middle_market.xlsx
+++ b/data/industry_study/generated_revision/top100_fidcs_middle_market.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" r:id="Rbdc9b91b8b9e4b91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 100 FIDCs" sheetId="2" r:id="Rcf9d4dfa11a643e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" r:id="R22c8410294fe49bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 100 FIDCs" sheetId="2" r:id="Rdc275bc4a1c34971"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Padroniza cores e regime de colocação no deck
</commit_message>
<xml_diff>
--- a/data/industry_study/generated_revision/top100_fidcs_middle_market.xlsx
+++ b/data/industry_study/generated_revision/top100_fidcs_middle_market.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" r:id="R22c8410294fe49bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 100 FIDCs" sheetId="2" r:id="Rdc275bc4a1c34971"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" r:id="R7f168d8075374616"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 100 FIDCs" sheetId="2" r:id="R1efeeda998644d87"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Amplia triagem de cedentes para Top 500 histórico
</commit_message>
<xml_diff>
--- a/data/industry_study/generated_revision/top100_fidcs_middle_market.xlsx
+++ b/data/industry_study/generated_revision/top100_fidcs_middle_market.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" r:id="R7f168d8075374616"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 100 FIDCs" sheetId="2" r:id="R1efeeda998644d87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" r:id="R15e678e7de6f4240"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 100 FIDCs" sheetId="2" r:id="R377a58c234e741ab"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>